<commit_message>
Remove unused Interfaces DESCRIPTION column from both templates
"DESCRIPTION" on the Interfaces sheet was already read and silently
dropped (the real interface schema has no field for it), so this
removes the column from both templates, their example-data workbooks,
and the test fixtures, and cleans up TemplateFlattener's docblock/
inline comments that documented the now-nonexistent drop. Output is
unaffected: verified byte-identical against the existing output_alt/
baseline and a fresh original-template build.
</commit_message>
<xml_diff>
--- a/Organization_Template.xlsx
+++ b/Organization_Template.xlsx
@@ -1655,7 +1655,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:I4"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10.5703125" bestFit="1" customWidth="1" style="23" min="1" max="1"/>
@@ -1706,11 +1706,6 @@
       </c>
       <c r="H2" s="32" t="inlineStr">
         <is>
-          <t>DESCRIPTION</t>
-        </is>
-      </c>
-      <c r="I2" s="32" t="inlineStr">
-        <is>
           <t>NOTES</t>
         </is>
       </c>
@@ -1721,7 +1716,6 @@
       <c r="D3" s="6" t="n"/>
       <c r="F3" s="25" t="n"/>
       <c r="G3" s="25" t="n"/>
-      <c r="H3" s="25" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="25" t="n"/>
@@ -1729,7 +1723,6 @@
       <c r="D4" s="25" t="n"/>
       <c r="F4" s="25" t="n"/>
       <c r="G4" s="25" t="n"/>
-      <c r="H4" s="25" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="2">

</xml_diff>